<commit_message>
feat: per-price unit economics for both products, P&L detail, simpler ParkinSense, kill/persevere thresholds, team mind map, founders as hardware & test engineers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpTS63SjPZxkBKCy56nCaA
</commit_message>
<xml_diff>
--- a/model/AVERRA_Financial_Model.xlsx
+++ b/model/AVERRA_Financial_Model.xlsx
@@ -1118,7 +1118,7 @@
     <t xml:space="preserve">ParkinSense RUO kit devices (5 × COGS per kit sold)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hardware &amp; test engineer</t>
+    <t xml:space="preserve">Hardware &amp; test engineering (done by the founders, no hire)</t>
   </si>
   <si>
     <t xml:space="preserve">ISO 13485 QMS set-up + surveillance audits</t>
@@ -4229,15 +4229,15 @@
       </c>
       <c r="B26" s="19" t="n">
         <f aca="false">IF(B24&lt;=0,"never",Forecast!$C$81/B24)</f>
-        <v>254.056965477916</v>
+        <v>226.81466525516</v>
       </c>
       <c r="C26" s="19" t="n">
         <f aca="false">IF(C24&lt;=0,"never",Forecast!$C$81/C24)</f>
-        <v>222.313246287427</v>
+        <v>198.474796562323</v>
       </c>
       <c r="D26" s="19" t="n">
         <f aca="false">IF(D24&lt;=0,"never",Forecast!$C$81/D24)</f>
-        <v>145.176839448618</v>
+        <v>129.609657347508</v>
       </c>
       <c r="E26" s="16" t="s">
         <v>190</v>
@@ -7296,98 +7296,98 @@
         <v>0</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="T16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="W16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="X16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="Y16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="Z16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AB16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AC16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AD16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AE16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AF16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AG16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AI16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AK16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AL16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AM16" s="4" t="n">
-        <v>55000</v>
+        <v>0</v>
       </c>
       <c r="AN16" s="22" t="n">
         <f aca="false">SUM(D16:O16)</f>
-        <v>330000</v>
+        <v>0</v>
       </c>
       <c r="AO16" s="22" t="n">
         <f aca="false">SUM(D16:I16)</f>
@@ -7395,15 +7395,15 @@
       </c>
       <c r="AP16" s="22" t="n">
         <f aca="false">SUM(J16:U16)</f>
-        <v>660000</v>
+        <v>0</v>
       </c>
       <c r="AQ16" s="22" t="n">
         <f aca="false">SUM(P16:AA16)</f>
-        <v>660000</v>
+        <v>0</v>
       </c>
       <c r="AR16" s="22" t="n">
         <f aca="false">SUM(AB16:AM16)</f>
-        <v>660000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9336,127 +9336,127 @@
       </c>
       <c r="J30" s="23" t="n">
         <f aca="false">SUM(J4:J29)</f>
-        <v>310000</v>
+        <v>255000</v>
       </c>
       <c r="K30" s="23" t="n">
         <f aca="false">SUM(K4:K29)</f>
-        <v>225000</v>
+        <v>170000</v>
       </c>
       <c r="L30" s="23" t="n">
         <f aca="false">SUM(L4:L29)</f>
-        <v>440000</v>
+        <v>385000</v>
       </c>
       <c r="M30" s="23" t="n">
         <f aca="false">SUM(M4:M29)</f>
-        <v>457650</v>
+        <v>402650</v>
       </c>
       <c r="N30" s="23" t="n">
         <f aca="false">SUM(N4:N29)</f>
-        <v>663036.9</v>
+        <v>608036.9</v>
       </c>
       <c r="O30" s="23" t="n">
         <f aca="false">SUM(O4:O29)</f>
-        <v>307650</v>
+        <v>252650</v>
       </c>
       <c r="P30" s="23" t="n">
         <f aca="false">SUM(P4:P29)</f>
-        <v>225000</v>
+        <v>170000</v>
       </c>
       <c r="Q30" s="23" t="n">
         <f aca="false">SUM(Q4:Q29)</f>
-        <v>242650</v>
+        <v>187650</v>
       </c>
       <c r="R30" s="23" t="n">
         <f aca="false">SUM(R4:R29)</f>
-        <v>466518.45</v>
+        <v>411518.45</v>
       </c>
       <c r="S30" s="23" t="n">
         <f aca="false">SUM(S4:S29)</f>
-        <v>484168.45</v>
+        <v>429168.45</v>
       </c>
       <c r="T30" s="23" t="n">
         <f aca="false">SUM(T4:T29)</f>
-        <v>466518.45</v>
+        <v>411518.45</v>
       </c>
       <c r="U30" s="23" t="n">
         <f aca="false">SUM(U4:U29)</f>
-        <v>1184168.45</v>
+        <v>1129168.45</v>
       </c>
       <c r="V30" s="23" t="n">
         <f aca="false">SUM(V4:V29)</f>
-        <v>520850</v>
+        <v>465850</v>
       </c>
       <c r="W30" s="23" t="n">
         <f aca="false">SUM(W4:W29)</f>
-        <v>534450</v>
+        <v>479450</v>
       </c>
       <c r="X30" s="23" t="n">
         <f aca="false">SUM(X4:X29)</f>
-        <v>548050</v>
+        <v>493050</v>
       </c>
       <c r="Y30" s="23" t="n">
         <f aca="false">SUM(Y4:Y29)</f>
-        <v>601650</v>
+        <v>546650</v>
       </c>
       <c r="Z30" s="23" t="n">
         <f aca="false">SUM(Z4:Z29)</f>
-        <v>575250</v>
+        <v>520250</v>
       </c>
       <c r="AA30" s="23" t="n">
         <f aca="false">SUM(AA4:AA29)</f>
-        <v>588850</v>
+        <v>533850</v>
       </c>
       <c r="AB30" s="23" t="n">
         <f aca="false">SUM(AB4:AB29)</f>
-        <v>1154010</v>
+        <v>1099010</v>
       </c>
       <c r="AC30" s="23" t="n">
         <f aca="false">SUM(AC4:AC29)</f>
-        <v>1218982</v>
+        <v>1163982</v>
       </c>
       <c r="AD30" s="23" t="n">
         <f aca="false">SUM(AD4:AD29)</f>
-        <v>1284060.4</v>
+        <v>1229060.4</v>
       </c>
       <c r="AE30" s="23" t="n">
         <f aca="false">SUM(AE4:AE29)</f>
-        <v>1349239.88</v>
+        <v>1294239.88</v>
       </c>
       <c r="AF30" s="23" t="n">
         <f aca="false">SUM(AF4:AF29)</f>
-        <v>1414515.386</v>
+        <v>1359515.386</v>
       </c>
       <c r="AG30" s="23" t="n">
         <f aca="false">SUM(AG4:AG29)</f>
-        <v>1519882.1167</v>
+        <v>1464882.1167</v>
       </c>
       <c r="AH30" s="23" t="n">
         <f aca="false">SUM(AH4:AH29)</f>
-        <v>1545335.510865</v>
+        <v>1490335.510865</v>
       </c>
       <c r="AI30" s="23" t="n">
         <f aca="false">SUM(AI4:AI29)</f>
-        <v>1610871.23532175</v>
+        <v>1555871.23532175</v>
       </c>
       <c r="AJ30" s="23" t="n">
         <f aca="false">SUM(AJ4:AJ29)</f>
-        <v>1676485.17355566</v>
+        <v>1621485.17355566</v>
       </c>
       <c r="AK30" s="23" t="n">
         <f aca="false">SUM(AK4:AK29)</f>
-        <v>1782173.41487788</v>
+        <v>1727173.41487788</v>
       </c>
       <c r="AL30" s="23" t="n">
         <f aca="false">SUM(AL4:AL29)</f>
-        <v>1807932.24413399</v>
+        <v>1752932.24413399</v>
       </c>
       <c r="AM30" s="23" t="n">
         <f aca="false">SUM(AM4:AM29)</f>
-        <v>1873758.13192729</v>
+        <v>1818758.13192729</v>
       </c>
       <c r="AN30" s="23" t="n">
         <f aca="false">SUM(D30:O30)</f>
-        <v>3199678.368</v>
+        <v>2869678.368</v>
       </c>
       <c r="AO30" s="23" t="n">
         <f aca="false">SUM(D30:I30)</f>
@@ -9464,15 +9464,15 @@
       </c>
       <c r="AP30" s="23" t="n">
         <f aca="false">SUM(J30:U30)</f>
-        <v>5472360.7</v>
+        <v>4812360.7</v>
       </c>
       <c r="AQ30" s="23" t="n">
         <f aca="false">SUM(P30:AA30)</f>
-        <v>6438123.8</v>
+        <v>5778123.8</v>
       </c>
       <c r="AR30" s="23" t="n">
         <f aca="false">SUM(AB30:AM30)</f>
-        <v>18237245.4933816</v>
+        <v>17577245.4933816</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9505,127 +9505,127 @@
       </c>
       <c r="J31" s="22" t="n">
         <f aca="false">J30*Assumptions!$C$35</f>
-        <v>31000</v>
+        <v>25500</v>
       </c>
       <c r="K31" s="22" t="n">
         <f aca="false">K30*Assumptions!$C$35</f>
-        <v>22500</v>
+        <v>17000</v>
       </c>
       <c r="L31" s="22" t="n">
         <f aca="false">L30*Assumptions!$C$35</f>
-        <v>44000</v>
+        <v>38500</v>
       </c>
       <c r="M31" s="22" t="n">
         <f aca="false">M30*Assumptions!$C$35</f>
-        <v>45765</v>
+        <v>40265</v>
       </c>
       <c r="N31" s="22" t="n">
         <f aca="false">N30*Assumptions!$C$35</f>
-        <v>66303.69</v>
+        <v>60803.69</v>
       </c>
       <c r="O31" s="22" t="n">
         <f aca="false">O30*Assumptions!$C$35</f>
-        <v>30765</v>
+        <v>25265</v>
       </c>
       <c r="P31" s="22" t="n">
         <f aca="false">P30*Assumptions!$C$35</f>
-        <v>22500</v>
+        <v>17000</v>
       </c>
       <c r="Q31" s="22" t="n">
         <f aca="false">Q30*Assumptions!$C$35</f>
-        <v>24265</v>
+        <v>18765</v>
       </c>
       <c r="R31" s="22" t="n">
         <f aca="false">R30*Assumptions!$C$35</f>
-        <v>46651.845</v>
+        <v>41151.845</v>
       </c>
       <c r="S31" s="22" t="n">
         <f aca="false">S30*Assumptions!$C$35</f>
-        <v>48416.845</v>
+        <v>42916.845</v>
       </c>
       <c r="T31" s="22" t="n">
         <f aca="false">T30*Assumptions!$C$35</f>
-        <v>46651.845</v>
+        <v>41151.845</v>
       </c>
       <c r="U31" s="22" t="n">
         <f aca="false">U30*Assumptions!$C$35</f>
-        <v>118416.845</v>
+        <v>112916.845</v>
       </c>
       <c r="V31" s="22" t="n">
         <f aca="false">V30*Assumptions!$C$35</f>
-        <v>52085</v>
+        <v>46585</v>
       </c>
       <c r="W31" s="22" t="n">
         <f aca="false">W30*Assumptions!$C$35</f>
-        <v>53445</v>
+        <v>47945</v>
       </c>
       <c r="X31" s="22" t="n">
         <f aca="false">X30*Assumptions!$C$35</f>
-        <v>54805</v>
+        <v>49305</v>
       </c>
       <c r="Y31" s="22" t="n">
         <f aca="false">Y30*Assumptions!$C$35</f>
-        <v>60165</v>
+        <v>54665</v>
       </c>
       <c r="Z31" s="22" t="n">
         <f aca="false">Z30*Assumptions!$C$35</f>
-        <v>57525</v>
+        <v>52025</v>
       </c>
       <c r="AA31" s="22" t="n">
         <f aca="false">AA30*Assumptions!$C$35</f>
-        <v>58885</v>
+        <v>53385</v>
       </c>
       <c r="AB31" s="22" t="n">
         <f aca="false">AB30*Assumptions!$C$35</f>
-        <v>115401</v>
+        <v>109901</v>
       </c>
       <c r="AC31" s="22" t="n">
         <f aca="false">AC30*Assumptions!$C$35</f>
-        <v>121898.2</v>
+        <v>116398.2</v>
       </c>
       <c r="AD31" s="22" t="n">
         <f aca="false">AD30*Assumptions!$C$35</f>
-        <v>128406.04</v>
+        <v>122906.04</v>
       </c>
       <c r="AE31" s="22" t="n">
         <f aca="false">AE30*Assumptions!$C$35</f>
-        <v>134923.988</v>
+        <v>129423.988</v>
       </c>
       <c r="AF31" s="22" t="n">
         <f aca="false">AF30*Assumptions!$C$35</f>
-        <v>141451.5386</v>
+        <v>135951.5386</v>
       </c>
       <c r="AG31" s="22" t="n">
         <f aca="false">AG30*Assumptions!$C$35</f>
-        <v>151988.21167</v>
+        <v>146488.21167</v>
       </c>
       <c r="AH31" s="22" t="n">
         <f aca="false">AH30*Assumptions!$C$35</f>
-        <v>154533.5510865</v>
+        <v>149033.5510865</v>
       </c>
       <c r="AI31" s="22" t="n">
         <f aca="false">AI30*Assumptions!$C$35</f>
-        <v>161087.123532175</v>
+        <v>155587.123532175</v>
       </c>
       <c r="AJ31" s="22" t="n">
         <f aca="false">AJ30*Assumptions!$C$35</f>
-        <v>167648.517355566</v>
+        <v>162148.517355566</v>
       </c>
       <c r="AK31" s="22" t="n">
         <f aca="false">AK30*Assumptions!$C$35</f>
-        <v>178217.341487788</v>
+        <v>172717.341487788</v>
       </c>
       <c r="AL31" s="22" t="n">
         <f aca="false">AL30*Assumptions!$C$35</f>
-        <v>180793.224413399</v>
+        <v>175293.224413399</v>
       </c>
       <c r="AM31" s="22" t="n">
         <f aca="false">AM30*Assumptions!$C$35</f>
-        <v>187375.813192729</v>
+        <v>181875.813192729</v>
       </c>
       <c r="AN31" s="23" t="n">
         <f aca="false">SUM(D31:O31)</f>
-        <v>319967.8368</v>
+        <v>286967.8368</v>
       </c>
       <c r="AO31" s="23" t="n">
         <f aca="false">SUM(D31:I31)</f>
@@ -9633,15 +9633,15 @@
       </c>
       <c r="AP31" s="23" t="n">
         <f aca="false">SUM(J31:U31)</f>
-        <v>547236.07</v>
+        <v>481236.07</v>
       </c>
       <c r="AQ31" s="23" t="n">
         <f aca="false">SUM(P31:AA31)</f>
-        <v>643812.38</v>
+        <v>577812.38</v>
       </c>
       <c r="AR31" s="23" t="n">
         <f aca="false">SUM(AB31:AM31)</f>
-        <v>1823724.54933816</v>
+        <v>1757724.54933816</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9674,127 +9674,127 @@
       </c>
       <c r="J32" s="23" t="n">
         <f aca="false">J30+J31</f>
-        <v>341000</v>
+        <v>280500</v>
       </c>
       <c r="K32" s="23" t="n">
         <f aca="false">K30+K31</f>
-        <v>247500</v>
+        <v>187000</v>
       </c>
       <c r="L32" s="23" t="n">
         <f aca="false">L30+L31</f>
-        <v>484000</v>
+        <v>423500</v>
       </c>
       <c r="M32" s="23" t="n">
         <f aca="false">M30+M31</f>
-        <v>503415</v>
+        <v>442915</v>
       </c>
       <c r="N32" s="23" t="n">
         <f aca="false">N30+N31</f>
-        <v>729340.59</v>
+        <v>668840.59</v>
       </c>
       <c r="O32" s="23" t="n">
         <f aca="false">O30+O31</f>
-        <v>338415</v>
+        <v>277915</v>
       </c>
       <c r="P32" s="23" t="n">
         <f aca="false">P30+P31</f>
-        <v>247500</v>
+        <v>187000</v>
       </c>
       <c r="Q32" s="23" t="n">
         <f aca="false">Q30+Q31</f>
-        <v>266915</v>
+        <v>206415</v>
       </c>
       <c r="R32" s="23" t="n">
         <f aca="false">R30+R31</f>
-        <v>513170.295</v>
+        <v>452670.295</v>
       </c>
       <c r="S32" s="23" t="n">
         <f aca="false">S30+S31</f>
-        <v>532585.295</v>
+        <v>472085.295</v>
       </c>
       <c r="T32" s="23" t="n">
         <f aca="false">T30+T31</f>
-        <v>513170.295</v>
+        <v>452670.295</v>
       </c>
       <c r="U32" s="23" t="n">
         <f aca="false">U30+U31</f>
-        <v>1302585.295</v>
+        <v>1242085.295</v>
       </c>
       <c r="V32" s="23" t="n">
         <f aca="false">V30+V31</f>
-        <v>572935</v>
+        <v>512435</v>
       </c>
       <c r="W32" s="23" t="n">
         <f aca="false">W30+W31</f>
-        <v>587895</v>
+        <v>527395</v>
       </c>
       <c r="X32" s="23" t="n">
         <f aca="false">X30+X31</f>
-        <v>602855</v>
+        <v>542355</v>
       </c>
       <c r="Y32" s="23" t="n">
         <f aca="false">Y30+Y31</f>
-        <v>661815</v>
+        <v>601315</v>
       </c>
       <c r="Z32" s="23" t="n">
         <f aca="false">Z30+Z31</f>
-        <v>632775</v>
+        <v>572275</v>
       </c>
       <c r="AA32" s="23" t="n">
         <f aca="false">AA30+AA31</f>
-        <v>647735</v>
+        <v>587235</v>
       </c>
       <c r="AB32" s="23" t="n">
         <f aca="false">AB30+AB31</f>
-        <v>1269411</v>
+        <v>1208911</v>
       </c>
       <c r="AC32" s="23" t="n">
         <f aca="false">AC30+AC31</f>
-        <v>1340880.2</v>
+        <v>1280380.2</v>
       </c>
       <c r="AD32" s="23" t="n">
         <f aca="false">AD30+AD31</f>
-        <v>1412466.44</v>
+        <v>1351966.44</v>
       </c>
       <c r="AE32" s="23" t="n">
         <f aca="false">AE30+AE31</f>
-        <v>1484163.868</v>
+        <v>1423663.868</v>
       </c>
       <c r="AF32" s="23" t="n">
         <f aca="false">AF30+AF31</f>
-        <v>1555966.9246</v>
+        <v>1495466.9246</v>
       </c>
       <c r="AG32" s="23" t="n">
         <f aca="false">AG30+AG31</f>
-        <v>1671870.32837</v>
+        <v>1611370.32837</v>
       </c>
       <c r="AH32" s="23" t="n">
         <f aca="false">AH30+AH31</f>
-        <v>1699869.0619515</v>
+        <v>1639369.0619515</v>
       </c>
       <c r="AI32" s="23" t="n">
         <f aca="false">AI30+AI31</f>
-        <v>1771958.35885393</v>
+        <v>1711458.35885393</v>
       </c>
       <c r="AJ32" s="23" t="n">
         <f aca="false">AJ30+AJ31</f>
-        <v>1844133.69091123</v>
+        <v>1783633.69091123</v>
       </c>
       <c r="AK32" s="23" t="n">
         <f aca="false">AK30+AK31</f>
-        <v>1960390.75636567</v>
+        <v>1899890.75636567</v>
       </c>
       <c r="AL32" s="23" t="n">
         <f aca="false">AL30+AL31</f>
-        <v>1988725.46854738</v>
+        <v>1928225.46854738</v>
       </c>
       <c r="AM32" s="23" t="n">
         <f aca="false">AM30+AM31</f>
-        <v>2061133.94512001</v>
+        <v>2000633.94512001</v>
       </c>
       <c r="AN32" s="23" t="n">
         <f aca="false">SUM(D32:O32)</f>
-        <v>3519646.2048</v>
+        <v>3156646.2048</v>
       </c>
       <c r="AO32" s="23" t="n">
         <f aca="false">SUM(D32:I32)</f>
@@ -9802,15 +9802,15 @@
       </c>
       <c r="AP32" s="23" t="n">
         <f aca="false">SUM(J32:U32)</f>
-        <v>6019596.77</v>
+        <v>5293596.77</v>
       </c>
       <c r="AQ32" s="23" t="n">
         <f aca="false">SUM(P32:AA32)</f>
-        <v>7081936.18</v>
+        <v>6355936.18</v>
       </c>
       <c r="AR32" s="23" t="n">
         <f aca="false">SUM(AB32:AM32)</f>
-        <v>20060970.0427197</v>
+        <v>19334970.0427197</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11414,127 +11414,127 @@
       </c>
       <c r="J45" s="22" t="n">
         <f aca="false">J43-J32</f>
-        <v>-341000</v>
+        <v>-280500</v>
       </c>
       <c r="K45" s="22" t="n">
         <f aca="false">K43-K32</f>
-        <v>-247500</v>
+        <v>-187000</v>
       </c>
       <c r="L45" s="22" t="n">
         <f aca="false">L43-L32</f>
-        <v>-484000</v>
+        <v>-423500</v>
       </c>
       <c r="M45" s="22" t="n">
         <f aca="false">M43-M32</f>
-        <v>-445106.525423729</v>
+        <v>-384606.525423729</v>
       </c>
       <c r="N45" s="22" t="n">
         <f aca="false">N43-N32</f>
-        <v>-729340.59</v>
+        <v>-668840.59</v>
       </c>
       <c r="O45" s="22" t="n">
         <f aca="false">O43-O32</f>
-        <v>-169582.239709443</v>
+        <v>-109082.239709443</v>
       </c>
       <c r="P45" s="22" t="n">
         <f aca="false">P43-P32</f>
-        <v>-63292.8571428572</v>
+        <v>-2792.85714285716</v>
       </c>
       <c r="Q45" s="22" t="n">
         <f aca="false">Q43-Q32</f>
-        <v>49283.4745762711</v>
+        <v>109783.474576271</v>
       </c>
       <c r="R45" s="22" t="n">
         <f aca="false">R43-R32</f>
-        <v>-144756.009285714</v>
+        <v>-84256.0092857142</v>
       </c>
       <c r="S45" s="22" t="n">
         <f aca="false">S43-S32</f>
-        <v>-105862.534709443</v>
+        <v>-45362.5347094431</v>
       </c>
       <c r="T45" s="22" t="n">
         <f aca="false">T43-T32</f>
-        <v>-144756.009285714</v>
+        <v>-84256.0092857142</v>
       </c>
       <c r="U45" s="22" t="n">
         <f aca="false">U43-U32</f>
-        <v>-875862.534709443</v>
+        <v>-815362.534709443</v>
       </c>
       <c r="V45" s="22" t="n">
         <f aca="false">V43-V32</f>
-        <v>-118243.668280872</v>
+        <v>-57743.6682808716</v>
       </c>
       <c r="W45" s="22" t="n">
         <f aca="false">W43-W32</f>
-        <v>-100171.763518967</v>
+        <v>-39671.7635189669</v>
       </c>
       <c r="X45" s="22" t="n">
         <f aca="false">X43-X32</f>
-        <v>-82099.8587570621</v>
+        <v>-21599.8587570621</v>
       </c>
       <c r="Y45" s="22" t="n">
         <f aca="false">Y43-Y32</f>
-        <v>-108027.953995157</v>
+        <v>-47527.9539951574</v>
       </c>
       <c r="Z45" s="22" t="n">
         <f aca="false">Z43-Z32</f>
-        <v>-45956.0492332527</v>
+        <v>14543.9507667474</v>
       </c>
       <c r="AA45" s="22" t="n">
         <f aca="false">AA43-AA32</f>
-        <v>-27884.1444713479</v>
+        <v>32615.8555286521</v>
       </c>
       <c r="AB45" s="22" t="n">
         <f aca="false">AB43-AB32</f>
-        <v>-17506.0524616628</v>
+        <v>42993.9475383372</v>
       </c>
       <c r="AC45" s="22" t="n">
         <f aca="false">AC43-AC32</f>
-        <v>3696.22857142845</v>
+        <v>64196.2285714285</v>
       </c>
       <c r="AD45" s="22" t="n">
         <f aca="false">AD43-AD32</f>
-        <v>25230.0628248588</v>
+        <v>85730.0628248588</v>
       </c>
       <c r="AE45" s="22" t="n">
         <f aca="false">AE43-AE32</f>
-        <v>47078.8726376111</v>
+        <v>107578.872637611</v>
       </c>
       <c r="AF45" s="22" t="n">
         <f aca="false">AF43-AF32</f>
-        <v>69226.9092317191</v>
+        <v>129726.909231719</v>
       </c>
       <c r="AG45" s="22" t="n">
         <f aca="false">AG43-AG32</f>
-        <v>47659.2112681158</v>
+        <v>108159.211268116</v>
       </c>
       <c r="AH45" s="22" t="n">
         <f aca="false">AH43-AH32</f>
-        <v>114361.565474685</v>
+        <v>174861.565474685</v>
       </c>
       <c r="AI45" s="22" t="n">
         <f aca="false">AI43-AI32</f>
-        <v>137320.46924292</v>
+        <v>197820.46924292</v>
       </c>
       <c r="AJ45" s="22" t="n">
         <f aca="false">AJ43-AJ32</f>
-        <v>160523.095094737</v>
+        <v>221023.095094737</v>
       </c>
       <c r="AK45" s="22" t="n">
         <f aca="false">AK43-AK32</f>
-        <v>139957.256925957</v>
+        <v>200457.256925957</v>
       </c>
       <c r="AL45" s="22" t="n">
         <f aca="false">AL43-AL32</f>
-        <v>207611.377937609</v>
+        <v>268111.377937609</v>
       </c>
       <c r="AM45" s="22" t="n">
         <f aca="false">AM43-AM32</f>
-        <v>231474.460170672</v>
+        <v>291974.460170672</v>
       </c>
       <c r="AN45" s="23" t="n">
         <f aca="false">SUM(D45:O45)</f>
-        <v>-3292504.96993317</v>
+        <v>-2929504.96993317</v>
       </c>
       <c r="AO45" s="23" t="n">
         <f aca="false">SUM(D45:I45)</f>
@@ -11542,15 +11542,15 @@
       </c>
       <c r="AP45" s="23" t="n">
         <f aca="false">SUM(J45:U45)</f>
-        <v>-3701775.82569007</v>
+        <v>-2975775.82569007</v>
       </c>
       <c r="AQ45" s="23" t="n">
         <f aca="false">SUM(P45:AA45)</f>
-        <v>-1767629.90881356</v>
+        <v>-1041629.90881356</v>
       </c>
       <c r="AR45" s="23" t="n">
         <f aca="false">SUM(AB45:AM45)</f>
-        <v>1166633.45691865</v>
+        <v>1892633.45691865</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11584,123 +11584,123 @@
       </c>
       <c r="J46" s="22" t="n">
         <f aca="false">J45+I46</f>
-        <v>-1216975.6148</v>
+        <v>-1156475.6148</v>
       </c>
       <c r="K46" s="22" t="n">
         <f aca="false">K45+J46</f>
-        <v>-1464475.6148</v>
+        <v>-1343475.6148</v>
       </c>
       <c r="L46" s="22" t="n">
         <f aca="false">L45+K46</f>
-        <v>-1948475.6148</v>
+        <v>-1766975.6148</v>
       </c>
       <c r="M46" s="22" t="n">
         <f aca="false">M45+L46</f>
-        <v>-2393582.14022373</v>
+        <v>-2151582.14022373</v>
       </c>
       <c r="N46" s="22" t="n">
         <f aca="false">N45+M46</f>
-        <v>-3122922.73022373</v>
+        <v>-2820422.73022373</v>
       </c>
       <c r="O46" s="22" t="n">
         <f aca="false">O45+N46</f>
-        <v>-3292504.96993317</v>
+        <v>-2929504.96993317</v>
       </c>
       <c r="P46" s="22" t="n">
         <f aca="false">P45+O46</f>
-        <v>-3355797.82707603</v>
+        <v>-2932297.82707603</v>
       </c>
       <c r="Q46" s="22" t="n">
         <f aca="false">Q45+P46</f>
-        <v>-3306514.35249976</v>
+        <v>-2822514.35249976</v>
       </c>
       <c r="R46" s="22" t="n">
         <f aca="false">R45+Q46</f>
-        <v>-3451270.36178547</v>
+        <v>-2906770.36178547</v>
       </c>
       <c r="S46" s="22" t="n">
         <f aca="false">S45+R46</f>
-        <v>-3557132.89649492</v>
+        <v>-2952132.89649492</v>
       </c>
       <c r="T46" s="22" t="n">
         <f aca="false">T45+S46</f>
-        <v>-3701888.90578063</v>
+        <v>-3036388.90578063</v>
       </c>
       <c r="U46" s="22" t="n">
         <f aca="false">U45+T46</f>
-        <v>-4577751.44049007</v>
+        <v>-3851751.44049007</v>
       </c>
       <c r="V46" s="22" t="n">
         <f aca="false">V45+U46</f>
-        <v>-4695995.10877094</v>
+        <v>-3909495.10877094</v>
       </c>
       <c r="W46" s="22" t="n">
         <f aca="false">W45+V46</f>
-        <v>-4796166.87228991</v>
+        <v>-3949166.87228991</v>
       </c>
       <c r="X46" s="22" t="n">
         <f aca="false">X45+W46</f>
-        <v>-4878266.73104697</v>
+        <v>-3970766.73104697</v>
       </c>
       <c r="Y46" s="22" t="n">
         <f aca="false">Y45+X46</f>
-        <v>-4986294.68504213</v>
+        <v>-4018294.68504213</v>
       </c>
       <c r="Z46" s="22" t="n">
         <f aca="false">Z45+Y46</f>
-        <v>-5032250.73427538</v>
+        <v>-4003750.73427538</v>
       </c>
       <c r="AA46" s="22" t="n">
         <f aca="false">AA45+Z46</f>
-        <v>-5060134.87874673</v>
+        <v>-3971134.87874673</v>
       </c>
       <c r="AB46" s="22" t="n">
         <f aca="false">AB45+AA46</f>
-        <v>-5077640.93120839</v>
+        <v>-3928140.93120839</v>
       </c>
       <c r="AC46" s="22" t="n">
         <f aca="false">AC45+AB46</f>
-        <v>-5073944.70263697</v>
+        <v>-3863944.70263697</v>
       </c>
       <c r="AD46" s="22" t="n">
         <f aca="false">AD45+AC46</f>
-        <v>-5048714.63981211</v>
+        <v>-3778214.63981211</v>
       </c>
       <c r="AE46" s="22" t="n">
         <f aca="false">AE45+AD46</f>
-        <v>-5001635.7671745</v>
+        <v>-3670635.7671745</v>
       </c>
       <c r="AF46" s="22" t="n">
         <f aca="false">AF45+AE46</f>
-        <v>-4932408.85794278</v>
+        <v>-3540908.85794278</v>
       </c>
       <c r="AG46" s="22" t="n">
         <f aca="false">AG45+AF46</f>
-        <v>-4884749.64667466</v>
+        <v>-3432749.64667466</v>
       </c>
       <c r="AH46" s="22" t="n">
         <f aca="false">AH45+AG46</f>
-        <v>-4770388.08119998</v>
+        <v>-3257888.08119998</v>
       </c>
       <c r="AI46" s="22" t="n">
         <f aca="false">AI45+AH46</f>
-        <v>-4633067.61195706</v>
+        <v>-3060067.61195705</v>
       </c>
       <c r="AJ46" s="22" t="n">
         <f aca="false">AJ45+AI46</f>
-        <v>-4472544.51686232</v>
+        <v>-2839044.51686232</v>
       </c>
       <c r="AK46" s="22" t="n">
         <f aca="false">AK45+AJ46</f>
-        <v>-4332587.25993636</v>
+        <v>-2638587.25993636</v>
       </c>
       <c r="AL46" s="22" t="n">
         <f aca="false">AL45+AK46</f>
-        <v>-4124975.88199875</v>
+        <v>-2370475.88199875</v>
       </c>
       <c r="AM46" s="22" t="n">
         <f aca="false">AM45+AL46</f>
-        <v>-3893501.42182808</v>
+        <v>-2078501.42182808</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11797,15 +11797,15 @@
       </c>
       <c r="Z47" s="22" t="n">
         <f aca="false">IF(AND(23&gt;=13,MIN(Z45:AM45)&gt;=0),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA47" s="22" t="n">
         <f aca="false">IF(AND(24&gt;=13,MIN(AA45:AM45)&gt;=0),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB47" s="22" t="n">
         <f aca="false">IF(AND(25&gt;=13,MIN(AB45:AM45)&gt;=0),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC47" s="22" t="n">
         <f aca="false">IF(AND(26&gt;=13,MIN(AC45:AM45)&gt;=0),1,0)</f>
@@ -11858,147 +11858,147 @@
       </c>
       <c r="D48" s="22" t="n">
         <f aca="false">D46+'Funding Scenarios'!$C$7+IF(1&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>3946869.11745007</v>
+        <v>2675653.62205056</v>
       </c>
       <c r="E48" s="22" t="n">
         <f aca="false">E46+'Funding Scenarios'!$C$7+IF(2&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>3754369.11745007</v>
+        <v>2483153.62205056</v>
       </c>
       <c r="F48" s="22" t="n">
         <f aca="false">F46+'Funding Scenarios'!$C$7+IF(3&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>5607693.50265007</v>
+        <v>4336478.00725056</v>
       </c>
       <c r="G48" s="22" t="n">
         <f aca="false">G46+'Funding Scenarios'!$C$7+IF(4&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>5448193.50265007</v>
+        <v>4176978.00725056</v>
       </c>
       <c r="H48" s="22" t="n">
         <f aca="false">H46+'Funding Scenarios'!$C$7+IF(5&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>5332693.50265007</v>
+        <v>4061478.00725056</v>
       </c>
       <c r="I48" s="22" t="n">
         <f aca="false">I46+'Funding Scenarios'!$C$7+IF(6&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>5217193.50265007</v>
+        <v>3945978.00725056</v>
       </c>
       <c r="J48" s="22" t="n">
         <f aca="false">J46+'Funding Scenarios'!$C$7+IF(7&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>4876193.50265007</v>
+        <v>3665478.00725056</v>
       </c>
       <c r="K48" s="22" t="n">
         <f aca="false">K46+'Funding Scenarios'!$C$7+IF(8&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>4628693.50265007</v>
+        <v>3478478.00725056</v>
       </c>
       <c r="L48" s="22" t="n">
         <f aca="false">L46+'Funding Scenarios'!$C$7+IF(9&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>4144693.50265007</v>
+        <v>3054978.00725056</v>
       </c>
       <c r="M48" s="22" t="n">
         <f aca="false">M46+'Funding Scenarios'!$C$7+IF(10&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>3699586.97722634</v>
+        <v>2670371.48182683</v>
       </c>
       <c r="N48" s="22" t="n">
         <f aca="false">N46+'Funding Scenarios'!$C$7+IF(11&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>2970246.38722634</v>
+        <v>2001530.89182683</v>
       </c>
       <c r="O48" s="22" t="n">
         <f aca="false">O46+'Funding Scenarios'!$C$7+IF(12&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>2800664.1475169</v>
+        <v>1892448.65211738</v>
       </c>
       <c r="P48" s="22" t="n">
         <f aca="false">P46+'Funding Scenarios'!$C$7+IF(13&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>2737371.29037404</v>
+        <v>1889655.79497453</v>
       </c>
       <c r="Q48" s="22" t="n">
         <f aca="false">Q46+'Funding Scenarios'!$C$7+IF(14&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>2786654.76495031</v>
+        <v>1999439.2695508</v>
       </c>
       <c r="R48" s="22" t="n">
         <f aca="false">R46+'Funding Scenarios'!$C$7+IF(15&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>2641898.7556646</v>
+        <v>1915183.26026508</v>
       </c>
       <c r="S48" s="22" t="n">
         <f aca="false">S46+'Funding Scenarios'!$C$7+IF(16&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>2536036.22095516</v>
+        <v>1869820.72555564</v>
       </c>
       <c r="T48" s="22" t="n">
         <f aca="false">T46+'Funding Scenarios'!$C$7+IF(17&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>2391280.21166944</v>
+        <v>1785564.71626993</v>
       </c>
       <c r="U48" s="22" t="n">
         <f aca="false">U46+'Funding Scenarios'!$C$7+IF(18&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1515417.67696</v>
+        <v>970202.181560484</v>
       </c>
       <c r="V48" s="22" t="n">
         <f aca="false">V46+'Funding Scenarios'!$C$7+IF(19&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1397174.00867913</v>
+        <v>912458.513279612</v>
       </c>
       <c r="W48" s="22" t="n">
         <f aca="false">W46+'Funding Scenarios'!$C$7+IF(20&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1297002.24516016</v>
+        <v>872786.749760645</v>
       </c>
       <c r="X48" s="22" t="n">
         <f aca="false">X46+'Funding Scenarios'!$C$7+IF(21&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1214902.3864031</v>
+        <v>851186.891003584</v>
       </c>
       <c r="Y48" s="22" t="n">
         <f aca="false">Y46+'Funding Scenarios'!$C$7+IF(22&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1106874.43240794</v>
+        <v>803658.937008426</v>
       </c>
       <c r="Z48" s="22" t="n">
         <f aca="false">Z46+'Funding Scenarios'!$C$7+IF(23&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1060918.38317469</v>
+        <v>818202.887775173</v>
       </c>
       <c r="AA48" s="22" t="n">
         <f aca="false">AA46+'Funding Scenarios'!$C$7+IF(24&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1033034.23870334</v>
+        <v>850818.743303826</v>
       </c>
       <c r="AB48" s="22" t="n">
         <f aca="false">AB46+'Funding Scenarios'!$C$7+IF(25&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1015528.18624168</v>
+        <v>893812.690842163</v>
       </c>
       <c r="AC48" s="22" t="n">
         <f aca="false">AC46+'Funding Scenarios'!$C$7+IF(26&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1019224.41481311</v>
+        <v>958008.919413591</v>
       </c>
       <c r="AD48" s="22" t="n">
         <f aca="false">AD46+'Funding Scenarios'!$C$7+IF(27&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1044454.47763796</v>
+        <v>1043738.98223845</v>
       </c>
       <c r="AE48" s="22" t="n">
         <f aca="false">AE46+'Funding Scenarios'!$C$7+IF(28&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1091533.35027558</v>
+        <v>1151317.85487606</v>
       </c>
       <c r="AF48" s="22" t="n">
         <f aca="false">AF46+'Funding Scenarios'!$C$7+IF(29&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1160760.25950729</v>
+        <v>1281044.76410778</v>
       </c>
       <c r="AG48" s="22" t="n">
         <f aca="false">AG46+'Funding Scenarios'!$C$7+IF(30&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1208419.47077541</v>
+        <v>1389203.9753759</v>
       </c>
       <c r="AH48" s="22" t="n">
         <f aca="false">AH46+'Funding Scenarios'!$C$7+IF(31&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1322781.03625009</v>
+        <v>1564065.54085058</v>
       </c>
       <c r="AI48" s="22" t="n">
         <f aca="false">AI46+'Funding Scenarios'!$C$7+IF(32&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1460101.50549302</v>
+        <v>1761886.0100935</v>
       </c>
       <c r="AJ48" s="22" t="n">
         <f aca="false">AJ46+'Funding Scenarios'!$C$7+IF(33&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1620624.60058775</v>
+        <v>1982909.10518824</v>
       </c>
       <c r="AK48" s="22" t="n">
         <f aca="false">AK46+'Funding Scenarios'!$C$7+IF(34&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1760581.85751371</v>
+        <v>2183366.3621142</v>
       </c>
       <c r="AL48" s="22" t="n">
         <f aca="false">AL46+'Funding Scenarios'!$C$7+IF(35&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>1968193.23545132</v>
+        <v>2451477.74005181</v>
       </c>
       <c r="AM48" s="22" t="n">
         <f aca="false">AM46+'Funding Scenarios'!$C$7+IF(36&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
-        <v>2199667.69562199</v>
+        <v>2743452.20022248</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12007,147 +12007,147 @@
       </c>
       <c r="D49" s="22" t="n">
         <f aca="false">D46+'Funding Scenarios'!$D$7</f>
-        <v>5946869.11745007</v>
+        <v>4675653.62205056</v>
       </c>
       <c r="E49" s="22" t="n">
         <f aca="false">E46+'Funding Scenarios'!$D$7</f>
-        <v>5754369.11745007</v>
+        <v>4483153.62205056</v>
       </c>
       <c r="F49" s="22" t="n">
         <f aca="false">F46+'Funding Scenarios'!$D$7</f>
-        <v>5607693.50265007</v>
+        <v>4336478.00725056</v>
       </c>
       <c r="G49" s="22" t="n">
         <f aca="false">G46+'Funding Scenarios'!$D$7</f>
-        <v>5448193.50265007</v>
+        <v>4176978.00725056</v>
       </c>
       <c r="H49" s="22" t="n">
         <f aca="false">H46+'Funding Scenarios'!$D$7</f>
-        <v>5332693.50265007</v>
+        <v>4061478.00725056</v>
       </c>
       <c r="I49" s="22" t="n">
         <f aca="false">I46+'Funding Scenarios'!$D$7</f>
-        <v>5217193.50265007</v>
+        <v>3945978.00725056</v>
       </c>
       <c r="J49" s="22" t="n">
         <f aca="false">J46+'Funding Scenarios'!$D$7</f>
-        <v>4876193.50265007</v>
+        <v>3665478.00725056</v>
       </c>
       <c r="K49" s="22" t="n">
         <f aca="false">K46+'Funding Scenarios'!$D$7</f>
-        <v>4628693.50265007</v>
+        <v>3478478.00725056</v>
       </c>
       <c r="L49" s="22" t="n">
         <f aca="false">L46+'Funding Scenarios'!$D$7</f>
-        <v>4144693.50265007</v>
+        <v>3054978.00725056</v>
       </c>
       <c r="M49" s="22" t="n">
         <f aca="false">M46+'Funding Scenarios'!$D$7</f>
-        <v>3699586.97722634</v>
+        <v>2670371.48182683</v>
       </c>
       <c r="N49" s="22" t="n">
         <f aca="false">N46+'Funding Scenarios'!$D$7</f>
-        <v>2970246.38722634</v>
+        <v>2001530.89182683</v>
       </c>
       <c r="O49" s="22" t="n">
         <f aca="false">O46+'Funding Scenarios'!$D$7</f>
-        <v>2800664.1475169</v>
+        <v>1892448.65211738</v>
       </c>
       <c r="P49" s="22" t="n">
         <f aca="false">P46+'Funding Scenarios'!$D$7</f>
-        <v>2737371.29037404</v>
+        <v>1889655.79497453</v>
       </c>
       <c r="Q49" s="22" t="n">
         <f aca="false">Q46+'Funding Scenarios'!$D$7</f>
-        <v>2786654.76495031</v>
+        <v>1999439.2695508</v>
       </c>
       <c r="R49" s="22" t="n">
         <f aca="false">R46+'Funding Scenarios'!$D$7</f>
-        <v>2641898.7556646</v>
+        <v>1915183.26026508</v>
       </c>
       <c r="S49" s="22" t="n">
         <f aca="false">S46+'Funding Scenarios'!$D$7</f>
-        <v>2536036.22095516</v>
+        <v>1869820.72555564</v>
       </c>
       <c r="T49" s="22" t="n">
         <f aca="false">T46+'Funding Scenarios'!$D$7</f>
-        <v>2391280.21166944</v>
+        <v>1785564.71626993</v>
       </c>
       <c r="U49" s="22" t="n">
         <f aca="false">U46+'Funding Scenarios'!$D$7</f>
-        <v>1515417.67696</v>
+        <v>970202.181560484</v>
       </c>
       <c r="V49" s="22" t="n">
         <f aca="false">V46+'Funding Scenarios'!$D$7</f>
-        <v>1397174.00867913</v>
+        <v>912458.513279612</v>
       </c>
       <c r="W49" s="22" t="n">
         <f aca="false">W46+'Funding Scenarios'!$D$7</f>
-        <v>1297002.24516016</v>
+        <v>872786.749760645</v>
       </c>
       <c r="X49" s="22" t="n">
         <f aca="false">X46+'Funding Scenarios'!$D$7</f>
-        <v>1214902.3864031</v>
+        <v>851186.891003584</v>
       </c>
       <c r="Y49" s="22" t="n">
         <f aca="false">Y46+'Funding Scenarios'!$D$7</f>
-        <v>1106874.43240794</v>
+        <v>803658.937008426</v>
       </c>
       <c r="Z49" s="22" t="n">
         <f aca="false">Z46+'Funding Scenarios'!$D$7</f>
-        <v>1060918.38317469</v>
+        <v>818202.887775173</v>
       </c>
       <c r="AA49" s="22" t="n">
         <f aca="false">AA46+'Funding Scenarios'!$D$7</f>
-        <v>1033034.23870334</v>
+        <v>850818.743303826</v>
       </c>
       <c r="AB49" s="22" t="n">
         <f aca="false">AB46+'Funding Scenarios'!$D$7</f>
-        <v>1015528.18624168</v>
+        <v>893812.690842163</v>
       </c>
       <c r="AC49" s="22" t="n">
         <f aca="false">AC46+'Funding Scenarios'!$D$7</f>
-        <v>1019224.41481311</v>
+        <v>958008.919413591</v>
       </c>
       <c r="AD49" s="22" t="n">
         <f aca="false">AD46+'Funding Scenarios'!$D$7</f>
-        <v>1044454.47763796</v>
+        <v>1043738.98223845</v>
       </c>
       <c r="AE49" s="22" t="n">
         <f aca="false">AE46+'Funding Scenarios'!$D$7</f>
-        <v>1091533.35027558</v>
+        <v>1151317.85487606</v>
       </c>
       <c r="AF49" s="22" t="n">
         <f aca="false">AF46+'Funding Scenarios'!$D$7</f>
-        <v>1160760.25950729</v>
+        <v>1281044.76410778</v>
       </c>
       <c r="AG49" s="22" t="n">
         <f aca="false">AG46+'Funding Scenarios'!$D$7</f>
-        <v>1208419.47077541</v>
+        <v>1389203.9753759</v>
       </c>
       <c r="AH49" s="22" t="n">
         <f aca="false">AH46+'Funding Scenarios'!$D$7</f>
-        <v>1322781.03625009</v>
+        <v>1564065.54085058</v>
       </c>
       <c r="AI49" s="22" t="n">
         <f aca="false">AI46+'Funding Scenarios'!$D$7</f>
-        <v>1460101.50549302</v>
+        <v>1761886.0100935</v>
       </c>
       <c r="AJ49" s="22" t="n">
         <f aca="false">AJ46+'Funding Scenarios'!$D$7</f>
-        <v>1620624.60058775</v>
+        <v>1982909.10518824</v>
       </c>
       <c r="AK49" s="22" t="n">
         <f aca="false">AK46+'Funding Scenarios'!$D$7</f>
-        <v>1760581.85751371</v>
+        <v>2183366.3621142</v>
       </c>
       <c r="AL49" s="22" t="n">
         <f aca="false">AL46+'Funding Scenarios'!$D$7</f>
-        <v>1968193.23545132</v>
+        <v>2451477.74005181</v>
       </c>
       <c r="AM49" s="22" t="n">
         <f aca="false">AM46+'Funding Scenarios'!$D$7</f>
-        <v>2199667.69562199</v>
+        <v>2743452.20022248</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12180,123 +12180,123 @@
       </c>
       <c r="J50" s="22" t="n">
         <f aca="false">J46+'Funding Scenarios'!$E$7</f>
-        <v>-165804.87704</v>
+        <v>-105304.87704</v>
       </c>
       <c r="K50" s="22" t="n">
         <f aca="false">K46+'Funding Scenarios'!$E$7</f>
-        <v>-413304.87704</v>
+        <v>-292304.87704</v>
       </c>
       <c r="L50" s="22" t="n">
         <f aca="false">L46+'Funding Scenarios'!$E$7</f>
-        <v>-897304.87704</v>
+        <v>-715804.87704</v>
       </c>
       <c r="M50" s="22" t="n">
         <f aca="false">M46+'Funding Scenarios'!$E$7</f>
-        <v>-1342411.40246373</v>
+        <v>-1100411.40246373</v>
       </c>
       <c r="N50" s="22" t="n">
         <f aca="false">N46+'Funding Scenarios'!$E$7</f>
-        <v>-2071751.99246373</v>
+        <v>-1769251.99246373</v>
       </c>
       <c r="O50" s="22" t="n">
         <f aca="false">O46+'Funding Scenarios'!$E$7</f>
-        <v>-2241334.23217317</v>
+        <v>-1878334.23217317</v>
       </c>
       <c r="P50" s="22" t="n">
         <f aca="false">P46+'Funding Scenarios'!$E$7</f>
-        <v>-2304627.08931603</v>
+        <v>-1881127.08931603</v>
       </c>
       <c r="Q50" s="22" t="n">
         <f aca="false">Q46+'Funding Scenarios'!$E$7</f>
-        <v>-2255343.61473976</v>
+        <v>-1771343.61473976</v>
       </c>
       <c r="R50" s="22" t="n">
         <f aca="false">R46+'Funding Scenarios'!$E$7</f>
-        <v>-2400099.62402547</v>
+        <v>-1855599.62402547</v>
       </c>
       <c r="S50" s="22" t="n">
         <f aca="false">S46+'Funding Scenarios'!$E$7</f>
-        <v>-2505962.15873492</v>
+        <v>-1900962.15873492</v>
       </c>
       <c r="T50" s="22" t="n">
         <f aca="false">T46+'Funding Scenarios'!$E$7</f>
-        <v>-2650718.16802063</v>
+        <v>-1985218.16802063</v>
       </c>
       <c r="U50" s="22" t="n">
         <f aca="false">U46+'Funding Scenarios'!$E$7</f>
-        <v>-3526580.70273007</v>
+        <v>-2800580.70273007</v>
       </c>
       <c r="V50" s="22" t="n">
         <f aca="false">V46+'Funding Scenarios'!$E$7</f>
-        <v>-3644824.37101094</v>
+        <v>-2858324.37101094</v>
       </c>
       <c r="W50" s="22" t="n">
         <f aca="false">W46+'Funding Scenarios'!$E$7</f>
-        <v>-3744996.13452991</v>
+        <v>-2897996.13452991</v>
       </c>
       <c r="X50" s="22" t="n">
         <f aca="false">X46+'Funding Scenarios'!$E$7</f>
-        <v>-3827095.99328697</v>
+        <v>-2919595.99328697</v>
       </c>
       <c r="Y50" s="22" t="n">
         <f aca="false">Y46+'Funding Scenarios'!$E$7</f>
-        <v>-3935123.94728213</v>
+        <v>-2967123.94728213</v>
       </c>
       <c r="Z50" s="22" t="n">
         <f aca="false">Z46+'Funding Scenarios'!$E$7</f>
-        <v>-3981079.99651538</v>
+        <v>-2952579.99651538</v>
       </c>
       <c r="AA50" s="22" t="n">
         <f aca="false">AA46+'Funding Scenarios'!$E$7</f>
-        <v>-4008964.14098673</v>
+        <v>-2919964.14098673</v>
       </c>
       <c r="AB50" s="22" t="n">
         <f aca="false">AB46+'Funding Scenarios'!$E$7</f>
-        <v>-4026470.19344839</v>
+        <v>-2876970.19344839</v>
       </c>
       <c r="AC50" s="22" t="n">
         <f aca="false">AC46+'Funding Scenarios'!$E$7</f>
-        <v>-4022773.96487696</v>
+        <v>-2812773.96487697</v>
       </c>
       <c r="AD50" s="22" t="n">
         <f aca="false">AD46+'Funding Scenarios'!$E$7</f>
-        <v>-3997543.90205211</v>
+        <v>-2727043.90205211</v>
       </c>
       <c r="AE50" s="22" t="n">
         <f aca="false">AE46+'Funding Scenarios'!$E$7</f>
-        <v>-3950465.0294145</v>
+        <v>-2619465.0294145</v>
       </c>
       <c r="AF50" s="22" t="n">
         <f aca="false">AF46+'Funding Scenarios'!$E$7</f>
-        <v>-3881238.12018278</v>
+        <v>-2489738.12018278</v>
       </c>
       <c r="AG50" s="22" t="n">
         <f aca="false">AG46+'Funding Scenarios'!$E$7</f>
-        <v>-3833578.90891466</v>
+        <v>-2381578.90891466</v>
       </c>
       <c r="AH50" s="22" t="n">
         <f aca="false">AH46+'Funding Scenarios'!$E$7</f>
-        <v>-3719217.34343998</v>
+        <v>-2206717.34343998</v>
       </c>
       <c r="AI50" s="22" t="n">
         <f aca="false">AI46+'Funding Scenarios'!$E$7</f>
-        <v>-3581896.87419706</v>
+        <v>-2008896.87419705</v>
       </c>
       <c r="AJ50" s="22" t="n">
         <f aca="false">AJ46+'Funding Scenarios'!$E$7</f>
-        <v>-3421373.77910232</v>
+        <v>-1787873.77910232</v>
       </c>
       <c r="AK50" s="22" t="n">
         <f aca="false">AK46+'Funding Scenarios'!$E$7</f>
-        <v>-3281416.52217636</v>
+        <v>-1587416.52217636</v>
       </c>
       <c r="AL50" s="22" t="n">
         <f aca="false">AL46+'Funding Scenarios'!$E$7</f>
-        <v>-3073805.14423875</v>
+        <v>-1319305.14423875</v>
       </c>
       <c r="AM50" s="22" t="n">
         <f aca="false">AM46+'Funding Scenarios'!$E$7</f>
-        <v>-2842330.68406808</v>
+        <v>-1027330.68406808</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12329,123 +12329,123 @@
       </c>
       <c r="J51" s="22" t="n">
         <f aca="false">J46+'Funding Scenarios'!$F$7</f>
-        <v>-165804.87704</v>
+        <v>-105304.87704</v>
       </c>
       <c r="K51" s="22" t="n">
         <f aca="false">K46+'Funding Scenarios'!$F$7</f>
-        <v>-413304.87704</v>
+        <v>-292304.87704</v>
       </c>
       <c r="L51" s="22" t="n">
         <f aca="false">L46+'Funding Scenarios'!$F$7</f>
-        <v>-897304.87704</v>
+        <v>-715804.87704</v>
       </c>
       <c r="M51" s="22" t="n">
         <f aca="false">M46+'Funding Scenarios'!$F$7</f>
-        <v>-1342411.40246373</v>
+        <v>-1100411.40246373</v>
       </c>
       <c r="N51" s="22" t="n">
         <f aca="false">N46+'Funding Scenarios'!$F$7</f>
-        <v>-2071751.99246373</v>
+        <v>-1769251.99246373</v>
       </c>
       <c r="O51" s="22" t="n">
         <f aca="false">O46+'Funding Scenarios'!$F$7</f>
-        <v>-2241334.23217317</v>
+        <v>-1878334.23217317</v>
       </c>
       <c r="P51" s="22" t="n">
         <f aca="false">P46+'Funding Scenarios'!$F$7</f>
-        <v>-2304627.08931603</v>
+        <v>-1881127.08931603</v>
       </c>
       <c r="Q51" s="22" t="n">
         <f aca="false">Q46+'Funding Scenarios'!$F$7</f>
-        <v>-2255343.61473976</v>
+        <v>-1771343.61473976</v>
       </c>
       <c r="R51" s="22" t="n">
         <f aca="false">R46+'Funding Scenarios'!$F$7</f>
-        <v>-2400099.62402547</v>
+        <v>-1855599.62402547</v>
       </c>
       <c r="S51" s="22" t="n">
         <f aca="false">S46+'Funding Scenarios'!$F$7</f>
-        <v>-2505962.15873492</v>
+        <v>-1900962.15873492</v>
       </c>
       <c r="T51" s="22" t="n">
         <f aca="false">T46+'Funding Scenarios'!$F$7</f>
-        <v>-2650718.16802063</v>
+        <v>-1985218.16802063</v>
       </c>
       <c r="U51" s="22" t="n">
         <f aca="false">U46+'Funding Scenarios'!$F$7</f>
-        <v>-3526580.70273007</v>
+        <v>-2800580.70273007</v>
       </c>
       <c r="V51" s="22" t="n">
         <f aca="false">V46+'Funding Scenarios'!$F$7</f>
-        <v>-3644824.37101094</v>
+        <v>-2858324.37101094</v>
       </c>
       <c r="W51" s="22" t="n">
         <f aca="false">W46+'Funding Scenarios'!$F$7</f>
-        <v>-3744996.13452991</v>
+        <v>-2897996.13452991</v>
       </c>
       <c r="X51" s="22" t="n">
         <f aca="false">X46+'Funding Scenarios'!$F$7</f>
-        <v>-3827095.99328697</v>
+        <v>-2919595.99328697</v>
       </c>
       <c r="Y51" s="22" t="n">
         <f aca="false">Y46+'Funding Scenarios'!$F$7</f>
-        <v>-3935123.94728213</v>
+        <v>-2967123.94728213</v>
       </c>
       <c r="Z51" s="22" t="n">
         <f aca="false">Z46+'Funding Scenarios'!$F$7</f>
-        <v>-3981079.99651538</v>
+        <v>-2952579.99651538</v>
       </c>
       <c r="AA51" s="22" t="n">
         <f aca="false">AA46+'Funding Scenarios'!$F$7</f>
-        <v>-4008964.14098673</v>
+        <v>-2919964.14098673</v>
       </c>
       <c r="AB51" s="22" t="n">
         <f aca="false">AB46+'Funding Scenarios'!$F$7</f>
-        <v>-4026470.19344839</v>
+        <v>-2876970.19344839</v>
       </c>
       <c r="AC51" s="22" t="n">
         <f aca="false">AC46+'Funding Scenarios'!$F$7</f>
-        <v>-4022773.96487696</v>
+        <v>-2812773.96487697</v>
       </c>
       <c r="AD51" s="22" t="n">
         <f aca="false">AD46+'Funding Scenarios'!$F$7</f>
-        <v>-3997543.90205211</v>
+        <v>-2727043.90205211</v>
       </c>
       <c r="AE51" s="22" t="n">
         <f aca="false">AE46+'Funding Scenarios'!$F$7</f>
-        <v>-3950465.0294145</v>
+        <v>-2619465.0294145</v>
       </c>
       <c r="AF51" s="22" t="n">
         <f aca="false">AF46+'Funding Scenarios'!$F$7</f>
-        <v>-3881238.12018278</v>
+        <v>-2489738.12018278</v>
       </c>
       <c r="AG51" s="22" t="n">
         <f aca="false">AG46+'Funding Scenarios'!$F$7</f>
-        <v>-3833578.90891466</v>
+        <v>-2381578.90891466</v>
       </c>
       <c r="AH51" s="22" t="n">
         <f aca="false">AH46+'Funding Scenarios'!$F$7</f>
-        <v>-3719217.34343998</v>
+        <v>-2206717.34343998</v>
       </c>
       <c r="AI51" s="22" t="n">
         <f aca="false">AI46+'Funding Scenarios'!$F$7</f>
-        <v>-3581896.87419706</v>
+        <v>-2008896.87419705</v>
       </c>
       <c r="AJ51" s="22" t="n">
         <f aca="false">AJ46+'Funding Scenarios'!$F$7</f>
-        <v>-3421373.77910232</v>
+        <v>-1787873.77910232</v>
       </c>
       <c r="AK51" s="22" t="n">
         <f aca="false">AK46+'Funding Scenarios'!$F$7</f>
-        <v>-3281416.52217636</v>
+        <v>-1587416.52217636</v>
       </c>
       <c r="AL51" s="22" t="n">
         <f aca="false">AL46+'Funding Scenarios'!$F$7</f>
-        <v>-3073805.14423875</v>
+        <v>-1319305.14423875</v>
       </c>
       <c r="AM51" s="22" t="n">
         <f aca="false">AM46+'Funding Scenarios'!$F$7</f>
-        <v>-2842330.68406808</v>
+        <v>-1027330.68406808</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13055,7 +13055,7 @@
       </c>
       <c r="D60" s="15" t="n">
         <f aca="false">AN32</f>
-        <v>3519646.2048</v>
+        <v>3156646.2048</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13073,7 +13073,7 @@
       </c>
       <c r="D62" s="15" t="n">
         <f aca="false">AN32/12</f>
-        <v>293303.8504</v>
+        <v>263053.8504</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13082,7 +13082,7 @@
       </c>
       <c r="D63" s="15" t="n">
         <f aca="false">-AN45/12</f>
-        <v>274375.414161098</v>
+        <v>244125.414161098</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="D66" s="15" t="n">
         <f aca="false">-MIN(D46:AM46)</f>
-        <v>5077640.93120839</v>
+        <v>4018294.68504213</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13118,8 +13118,8 @@
       </c>
       <c r="D67" s="24" t="str">
         <f aca="false">INDEX($D$3:$AM$3,MATCH(-D66,D46:AM46,0))</f>
-        <v>M25
-Jul-29</v>
+        <v>M22
+Apr-29</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13128,7 +13128,7 @@
       </c>
       <c r="D68" s="15" t="n">
         <f aca="false">D66*(1+Assumptions!$C$36)</f>
-        <v>6093169.11745007</v>
+        <v>4821953.62205056</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="D70" s="15" t="n">
         <f aca="false">D68-D69</f>
-        <v>5041998.37969007</v>
+        <v>3770782.88429056</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13155,8 +13155,8 @@
       </c>
       <c r="D71" s="24" t="str">
         <f aca="false">IFERROR(INDEX($D$3:$AM$3,MATCH(1,D47:AM47,0)),"Not within 36 months")</f>
-        <v>M26
-Aug-29</v>
+        <v>M23
+May-29</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13174,7 +13174,7 @@
       </c>
       <c r="D73" s="15" t="n">
         <f aca="false">AQ45</f>
-        <v>-1767629.90881356</v>
+        <v>-1041629.90881356</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13192,7 +13192,7 @@
       </c>
       <c r="D75" s="15" t="n">
         <f aca="false">AR45</f>
-        <v>1166633.45691865</v>
+        <v>1892633.45691865</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13201,7 +13201,7 @@
       </c>
       <c r="D76" s="25" t="n">
         <f aca="false">IF(D74=0,0,D75/D74)</f>
-        <v>0.0549583214581206</v>
+        <v>0.0891590733240752</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="D77" s="15" t="n">
         <f aca="false">AM45</f>
-        <v>231474.460170672</v>
+        <v>291974.460170672</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13219,7 +13219,7 @@
       </c>
       <c r="D78" s="15" t="n">
         <f aca="false">SUMIF($B$4:$B$29,"Shared",$AN$4:$AN$29)</f>
-        <v>1683000</v>
+        <v>1353000</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13246,11 +13246,11 @@
       </c>
       <c r="C81" s="14" t="n">
         <f aca="false">D81</f>
-        <v>564212.503559976</v>
+        <v>503712.503559976</v>
       </c>
       <c r="D81" s="15" t="n">
         <f aca="false">(AR32-(AR20+AR27+AR28+AR26)*(1+Assumptions!$C$35))/12</f>
-        <v>564212.503559976</v>
+        <v>503712.503559976</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13259,7 +13259,7 @@
       </c>
       <c r="D82" s="15" t="n">
         <f aca="false">(SUM(J32:O32)-SUM(J19:O19)*(1+Assumptions!$C$35))/6</f>
-        <v>352055</v>
+        <v>291555</v>
       </c>
     </row>
   </sheetData>
@@ -13470,19 +13470,19 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="n">
         <f aca="false">'Funding Scenarios'!C7</f>
-        <v>4093169.11745007</v>
+        <v>2821953.62205056</v>
       </c>
       <c r="B14" s="14" t="n">
         <f aca="false">A14*(1-Assumptions!$C$41)/Assumptions!$C$41</f>
-        <v>23194624.9988837</v>
+        <v>15991070.5249532</v>
       </c>
       <c r="C14" s="14" t="n">
         <f aca="false">A14*(1-Assumptions!$C$42)/Assumptions!$C$42</f>
-        <v>16372676.4698003</v>
+        <v>11287814.4882022</v>
       </c>
       <c r="D14" s="18" t="n">
         <f aca="false">IF(A14=0,0,A14/($F$10+A14))</f>
-        <v>0.353067317140144</v>
+        <v>0.273393363832025</v>
       </c>
       <c r="E14" s="3" t="str">
         <f aca="false">IF(D14&lt;=Assumptions!$C$41,"Within 15% at proposed P",IF(D14&lt;=Assumptions!$C$42,"Within 15–20% at proposed P","Above 20% at proposed P"))</f>
@@ -13492,19 +13492,19 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="n">
         <f aca="false">'Funding Scenarios'!D7</f>
-        <v>6093169.11745007</v>
+        <v>4821953.62205056</v>
       </c>
       <c r="B15" s="14" t="n">
         <f aca="false">A15*(1-Assumptions!$C$41)/Assumptions!$C$41</f>
-        <v>34527958.3322171</v>
+        <v>27324403.8582865</v>
       </c>
       <c r="C15" s="14" t="n">
         <f aca="false">A15*(1-Assumptions!$C$42)/Assumptions!$C$42</f>
-        <v>24372676.4698003</v>
+        <v>19287814.4882022</v>
       </c>
       <c r="D15" s="18" t="n">
         <f aca="false">IF(A15=0,0,A15/($F$10+A15))</f>
-        <v>0.448252285011892</v>
+        <v>0.391330284949418</v>
       </c>
       <c r="E15" s="3" t="str">
         <f aca="false">IF(D15&lt;=Assumptions!$C$41,"Within 15% at proposed P",IF(D15&lt;=Assumptions!$C$42,"Within 15–20% at proposed P","Above 20% at proposed P"))</f>
@@ -13701,11 +13701,11 @@
       </c>
       <c r="C4" s="28" t="n">
         <f aca="false">Forecast!$D$68</f>
-        <v>6093169.11745007</v>
+        <v>4821953.62205056</v>
       </c>
       <c r="D4" s="28" t="n">
         <f aca="false">Forecast!$D$68</f>
-        <v>6093169.11745007</v>
+        <v>4821953.62205056</v>
       </c>
       <c r="E4" s="28" t="n">
         <f aca="false">Forecast!$D$69</f>
@@ -13757,11 +13757,11 @@
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C4-C6</f>
-        <v>4093169.11745007</v>
+        <v>2821953.62205056</v>
       </c>
       <c r="D7" s="28" t="n">
         <f aca="false">D4-D6</f>
-        <v>6093169.11745007</v>
+        <v>4821953.62205056</v>
       </c>
       <c r="E7" s="28" t="n">
         <f aca="false">E4-E6</f>
@@ -13799,11 +13799,11 @@
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C8+C7</f>
-        <v>11593169.1174501</v>
+        <v>10321953.6220506</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">D8+D7</f>
-        <v>13593169.1174501</v>
+        <v>12321953.6220506</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">E8+E7</f>
@@ -13820,11 +13820,11 @@
       </c>
       <c r="C10" s="31" t="n">
         <f aca="false">C7/C9</f>
-        <v>0.353067317140144</v>
+        <v>0.273393363832025</v>
       </c>
       <c r="D10" s="31" t="n">
         <f aca="false">D7/D9</f>
-        <v>0.448252285011892</v>
+        <v>0.391330284949418</v>
       </c>
       <c r="E10" s="31" t="n">
         <f aca="false">E7/E9</f>
@@ -13862,11 +13862,11 @@
       </c>
       <c r="C12" s="31" t="n">
         <f aca="false">1-C10-C11</f>
-        <v>0.596932682859856</v>
+        <v>0.676606636167975</v>
       </c>
       <c r="D12" s="31" t="n">
         <f aca="false">1-D10-D11</f>
-        <v>0.501747714988108</v>
+        <v>0.558669715050582</v>
       </c>
       <c r="E12" s="31" t="n">
         <f aca="false">1-E10-E11</f>
@@ -13934,13 +13934,13 @@
       </c>
       <c r="C16" s="32" t="str">
         <f aca="false">IFERROR(INDEX(Forecast!$D$3:$AM$3,MATCH(1,Forecast!$D$52:$AM$52,0)),"Never — reaches break-even "&amp;Forecast!$D$71)</f>
-        <v>Never — reaches break-even M26
-Aug-29</v>
+        <v>Never — reaches break-even M23
+May-29</v>
       </c>
       <c r="D16" s="32" t="str">
         <f aca="false">IFERROR(INDEX(Forecast!$D$3:$AM$3,MATCH(1,Forecast!$D$53:$AM$53,0)),"Never — reaches break-even "&amp;Forecast!$D$71)</f>
-        <v>Never — reaches break-even M26
-Aug-29</v>
+        <v>Never — reaches break-even M23
+May-29</v>
       </c>
       <c r="E16" s="32" t="str">
         <f aca="false">IFERROR(INDEX(Forecast!$D$3:$AM$3,MATCH(1,Forecast!$D$54:$AM$54,0)),"Never — reaches break-even "&amp;Forecast!$D$71)</f>
@@ -13964,7 +13964,7 @@
       </c>
       <c r="F18" s="14" t="n">
         <f aca="false">Forecast!$D$70</f>
-        <v>5041998.37969007</v>
+        <v>3770782.88429056</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13981,7 +13981,7 @@
       </c>
       <c r="F20" s="14" t="n">
         <f aca="false">F18-F19</f>
-        <v>5041998.37969007</v>
+        <v>3770782.88429056</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13999,7 +13999,7 @@
       </c>
       <c r="F22" s="18" t="n">
         <f aca="false">F20/(F21+F20)</f>
-        <v>0.348465543264076</v>
+        <v>0.285710191092855</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14008,7 +14008,7 @@
       </c>
       <c r="F23" s="18" t="n">
         <f aca="false">F12*(1-F22)</f>
-        <v>0.538866483640386</v>
+        <v>0.59076973388986</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14017,7 +14017,7 @@
       </c>
       <c r="F24" s="18" t="n">
         <f aca="false">1-F23-F11*(1-F22)</f>
-        <v>0.428556793522818</v>
+        <v>0.373515775664782</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14081,7 +14081,7 @@
       </c>
       <c r="C4" s="17" t="n">
         <f aca="false">Forecast!AP4+Forecast!AP5+Forecast!AP16+Forecast!AP23+Forecast!AP24+Forecast!AP25</f>
-        <v>1380000</v>
+        <v>720000</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>503</v>
@@ -14177,7 +14177,7 @@
       </c>
       <c r="C10" s="17" t="n">
         <f aca="false">Forecast!AP31</f>
-        <v>547236.07</v>
+        <v>481236.07</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14190,7 +14190,7 @@
       </c>
       <c r="C11" s="15" t="n">
         <f aca="false">SUM(C4:C10)</f>
-        <v>6019596.77</v>
+        <v>5293596.77</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Competitors: Helio Strap at ₹12,000–15,000 with 10-day battery; restore ParkinSense price wording; latest prices; TremoSense demo video
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpTS63SjPZxkBKCy56nCaA
</commit_message>
<xml_diff>
--- a/model/AVERRA_Financial_Model.xlsx
+++ b/model/AVERRA_Financial_Model.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="604">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="608">
   <si>
     <t xml:space="preserve">AVERRA — model inputs (blue = input · yellow = key assumption to confirm · black = formula)</t>
   </si>
@@ -185,7 +185,7 @@
     <t xml:space="preserve">ParkinSense wellness wearable price (incl. GST)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hypothesis to test; below Amazfit Bip 6 (₹8,999) and Fitbit Charge 6 (₹12,999); positive contribution after CAC</t>
+    <t xml:space="preserve">Hypothesis to test; below Amazfit Helio Strap (₹12,000+), Google Fitbit Air (₹13,999), WHOOP One (₹20,890/yr) and Garmin Cirqa (₹25,990); positive contribution after CAC</t>
   </si>
   <si>
     <t xml:space="preserve">P4</t>
@@ -1646,16 +1646,16 @@
     <t xml:space="preserve">WHOOP One (WHOOP 5.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">Wellness wearable</t>
+    <t xml:space="preserve">Screenless band</t>
   </si>
   <si>
     <t xml:space="preserve">INR</t>
   </si>
   <si>
-    <t xml:space="preserve">Membership is the price: ₹17,990 / 12 months (MRP ₹21,990)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screenless strap; recovery, sleep, strain, steps, VO2 max; 14+ day battery</t>
+    <t xml:space="preserve">Price includes a 12-month membership (MRP ₹21,990); renews yearly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screenless strap; recovery, sleep, strain, HRV; 14+ day battery</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.whoop.in/pages/whoop-devices</t>
@@ -1664,135 +1664,141 @@
     <t xml:space="preserve">12 Oct 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">WHOOP Peak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">₹23,990 / 12 months (MRP ₹28,990)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adds healthspan, health monitor alerts, real-time stress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amazfit Bip 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fitness smartwatch</t>
+    <t xml:space="preserve">Garmin Cirqa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No subscription needed; Connect+ optional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR, HRV, Pulse Ox, sleep, VO2 max, skin temperature, 80+ activities; up to 10 days (launched in India 7 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.businesstoday.in/technology/news/story/garmin-cirqa-launched-in-india-at-rs25990-this-screen-free-smart-band-can-track-80-activities-560058-2026-10-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazfit Helio Strap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No subscription needed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Continuous HR, sleep and recovery (BioCharge), 27 exercise modes; up to 10 days. Available from sellers at ₹12,000–15,000; official store lists ₹8,999 (MRP ₹17,999) but shows sold out (16 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://in.amazfit.com/products/helio-strap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Fitbit Air</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-month Google Health Premium trial, then optional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR, HRV, SpO2, sleep stages, irregular-rhythm alerts; up to 7 days (India from 2 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.freepressjournal.in/tech/google-fitbit-air-launched-in-india-at-13999-price-specifications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GyroGlove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hand stabiliser (one hand)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Or $246/month × 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gyroscopic wrist stabiliser for the whole hand; 4 h continuous use; no clinical study cited on listing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://techguide.parkinsons.org.uk/catalogue/gyro-glove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imported active spoon (desertcart.in)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active stabilising utensil</t>
   </si>
   <si>
     <t xml:space="preserve">None listed</t>
   </si>
   <si>
-    <t xml:space="preserve">AMOLED, GPS, heart rate, sleep; accelerometer + gyroscope; up to 14 days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.91mobiles.com/amazfit-bip-6-smart-watch-price-in-india</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fitbit Charge 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fitness band</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional premium subscription (not priced here)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heart rate, SpO2, sleep, GPS; ~7 days (₹13,999 on Amazon)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.smartprix.com/fitness_bands/fitbit-charge-6-fitness-band-ppd10ccze2vi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GyroGlove</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hand stabiliser (one hand)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Or $246/month × 24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gyroscopic wrist stabiliser for the whole hand; 4 h continuous use; no clinical study cited on listing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://techguide.parkinsons.org.uk/catalogue/gyro-glove</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liftware (stabilising handle)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Active stabilising utensil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attachments extra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensor + motor cancellation at the utensil; maker cites a study with 70% less shaking. Price is a DATED Nov 2015 figure</t>
+    <t xml:space="preserve">Motorised stabilising spoon for essential tremor, imported; listing price in India (desertcart.in, checked 16 Oct 2026); similar listings ₹35,980 to ₹1,40,386</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.desertcart.in/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted soup spoon (225 g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passive adaptive utensil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added mass damps tremor; no electronics. US retail; Indian prices not verified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://wellbefore.com/products/weighted-soup-spoon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steady Spoon (imported, desertcart.in)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stabilising spoon handle, imported; lowest active-spoon listing found in India (desertcart.in, checked 16 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVERRA planned prices (to be tested with customers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TremoSense launch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TremoSense vs GyroGlove (one glove)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Different products: spoon stabiliser vs whole-hand glove — price context only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sources</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNFPA India Ageing Report 2023 (149M aged 60+, 10.5%; 347M by 2050)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.thenationalnews.com/world/asia/2023/09/28/india-un-elderly-population/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khurana &amp; Gourie-Devi, Cureus 2025;17(3):e80248 — Indian PD community studies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC11890171</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chin et al., Mov Disord 2021 — ET in rural Gujarat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mdsabstracts.org/abstract/prevalence-of-essential-tremors-in-rural-gujarat-india/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BMJ 2025 — PD prevalence 25.2M by 2050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://bmjgroup.com/cases-of-parkinsons-disease-set-to-reach-25-million-worldwide-by-2050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michael J. Fox Foundation — Liftware $195 (Nov 2015)</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.michaeljfox.org/news/stabilizing-spoon-announces-price-reduction-and-match-program-holidays</t>
   </si>
   <si>
-    <t xml:space="preserve">Weighted soup spoon (225 g)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passive adaptive utensil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Added mass damps tremor; no electronics. US retail; Indian prices not verified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://wellbefore.com/products/weighted-soup-spoon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVERRA price hypotheses (to be tested with customers)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TremoSense launch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TremoSense vs GyroGlove (one glove)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Different products: spoon stabiliser vs whole-hand glove — price context only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sources</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNFPA India Ageing Report 2023 (149M aged 60+, 10.5%; 347M by 2050)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.thenationalnews.com/world/asia/2023/09/28/india-un-elderly-population/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khurana &amp; Gourie-Devi, Cureus 2025;17(3):e80248 — Indian PD community studies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC11890171</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chin et al., Mov Disord 2021 — ET in rural Gujarat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.mdsabstracts.org/abstract/prevalence-of-essential-tremors-in-rural-gujarat-india/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BMJ 2025 — PD prevalence 25.2M by 2050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://bmjgroup.com/cases-of-parkinsons-disease-set-to-reach-25-million-worldwide-by-2050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michael J. Fox Foundation — Liftware $195 (Nov 2015)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Seeed Studio — XIAO nRF52840 Sense $15.90 / $13.90 (10+)</t>
   </si>
   <si>
@@ -1847,13 +1853,19 @@
     <t xml:space="preserve">https://tradersunion.com/currencies/price/usd-inr/</t>
   </si>
   <si>
-    <t xml:space="preserve">WHOOP India memberships (checked 12 Oct 2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amazfit Bip 6 India price (checked 12 Oct 2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fitbit Charge 6 India price (checked 12 Oct 2026)</t>
+    <t xml:space="preserve">WHOOP India memberships: One ₹20,890, Peak ₹27,539 (checked 16 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Garmin Cirqa India launch, ₹25,990 (Business Today, 7 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazfit Helio Strap India: official ₹8,999 (MRP ₹17,999), sold out; sellers ₹12,000–15,000 (16 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Fitbit Air India launch, ₹13,999 (Free Press Journal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imported active tremor spoons on desertcart.in: ₹35,980, ₹58,480, ₹1,40,386 (Google Shopping, checked 16 Oct 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">GyroGlove listing, Parkinson's UK tech guide (16 Jun 2026)</t>
@@ -3390,14 +3402,14 @@
         <v>526</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>17990</v>
+        <v>20890</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>527</v>
       </c>
       <c r="E4" s="14" t="n">
         <f aca="false">C4</f>
-        <v>17990</v>
+        <v>20890</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>528</v>
@@ -3420,14 +3432,14 @@
         <v>526</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>23990</v>
+        <v>25990</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>527</v>
       </c>
       <c r="E5" s="14" t="n">
         <f aca="false">C5</f>
-        <v>23990</v>
+        <v>25990</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>533</v>
@@ -3436,7 +3448,7 @@
         <v>534</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>530</v>
+        <v>535</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>531</v>
@@ -3444,20 +3456,20 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>536</v>
+        <v>526</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>8999</v>
+        <v>12000</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>527</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">C6</f>
-        <v>8999</v>
+        <v>12000</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>537</v>
@@ -3477,26 +3489,26 @@
         <v>540</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>541</v>
+        <v>526</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>12999</v>
+        <v>13999</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>527</v>
       </c>
       <c r="E7" s="14" t="n">
         <f aca="false">C7</f>
-        <v>12999</v>
+        <v>13999</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>542</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>543</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>544</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>531</v>
@@ -3504,29 +3516,29 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>545</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>546</v>
       </c>
       <c r="C8" s="34" t="n">
         <v>5899</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">C8*Assumptions!$C$40</f>
         <v>564593.29</v>
       </c>
       <c r="F8" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>548</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>549</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>550</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>531</v>
@@ -3534,29 +3546,29 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>551</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="11" t="n">
+        <v>58480</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <f aca="false">C9</f>
+        <v>58480</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>552</v>
       </c>
-      <c r="C9" s="34" t="n">
-        <v>195</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>547</v>
-      </c>
-      <c r="E9" s="14" t="n">
-        <f aca="false">C9*Assumptions!$C$40</f>
-        <v>18663.45</v>
-      </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>553</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>554</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>555</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>531</v>
@@ -3564,42 +3576,72 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>556</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>557</v>
       </c>
       <c r="C10" s="34" t="n">
         <v>55.98</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="E10" s="14" t="n">
         <f aca="false">C10*Assumptions!$C$40</f>
         <v>5357.8458</v>
       </c>
       <c r="F10" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>558</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>559</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>560</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>531</v>
       </c>
     </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>35980</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <f aca="false">C11</f>
+        <v>35980</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>561</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>531</v>
+      </c>
+    </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E13" s="17" t="n">
         <f aca="false">Assumptions!$C$12</f>
@@ -3617,14 +3659,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="E15" s="18" t="n">
         <f aca="false">E13/E8</f>
         <v>0.0177100935790434</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
   </sheetData>
@@ -3643,7 +3685,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="80"/>
@@ -3652,124 +3694,124 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>555</v>
+        <v>576</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>530</v>
@@ -3777,58 +3819,74 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>544</v>
+        <v>539</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>550</v>
+        <v>543</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>598</v>
+        <v>554</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>560</v>
+        <v>549</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>603</v>
+        <v>559</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>606</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>607</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Market: show general-wearable SOM as a range (0.25% plan, 0.5% and 1% upside)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpTS63SjPZxkBKCy56nCaA
</commit_message>
<xml_diff>
--- a/model/AVERRA_Financial_Model.xlsx
+++ b/model/AVERRA_Financial_Model.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="608">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="615">
   <si>
     <t xml:space="preserve">AVERRA — model inputs (blue = input · yellow = key assumption to confirm · black = formula)</t>
   </si>
@@ -897,6 +897,27 @@
   </si>
   <si>
     <t xml:space="preserve">ASSUMPTION: 0.25% of premium buyers via online channel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General-wearable SOM range (Year 3, upside only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOM share of SAM buyers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers / year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upside: marketing works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strong upside</t>
   </si>
   <si>
     <t xml:space="preserve">Monthly cash plan — Phase 1 PROVE (M1–M6) → Phase 2 LAUNCH (M7–M18) → SCALE (M19–M36). M1 = July 2027</t>
@@ -3362,286 +3383,286 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>517</v>
+        <v>524</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>519</v>
+        <v>526</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>521</v>
+        <v>528</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>522</v>
+        <v>529</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="C4" s="11" t="n">
         <v>20890</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="E4" s="14" t="n">
         <f aca="false">C4</f>
         <v>20890</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="C5" s="11" t="n">
         <v>25990</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="E5" s="14" t="n">
         <f aca="false">C5</f>
         <v>25990</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>536</v>
+        <v>543</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="C6" s="11" t="n">
         <v>12000</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">C6</f>
         <v>12000</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
       <c r="G6" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>538</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>539</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="C7" s="11" t="n">
         <v>13999</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="E7" s="14" t="n">
         <f aca="false">C7</f>
         <v>13999</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>541</v>
+        <v>548</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>543</v>
+        <v>550</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>545</v>
+        <v>552</v>
       </c>
       <c r="C8" s="34" t="n">
         <v>5899</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">C8*Assumptions!$C$40</f>
         <v>564593.29</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>550</v>
+        <v>557</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>551</v>
+        <v>558</v>
       </c>
       <c r="C9" s="11" t="n">
         <v>58480</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="E9" s="14" t="n">
         <f aca="false">C9</f>
         <v>58480</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>556</v>
+        <v>563</v>
       </c>
       <c r="C10" s="34" t="n">
         <v>55.98</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="E10" s="14" t="n">
         <f aca="false">C10*Assumptions!$C$40</f>
         <v>5357.8458</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>559</v>
+        <v>566</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>551</v>
+        <v>558</v>
       </c>
       <c r="C11" s="11" t="n">
         <v>35980</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="E11" s="14" t="n">
         <f aca="false">C11</f>
         <v>35980</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
       <c r="G11" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>561</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>554</v>
-      </c>
       <c r="I11" s="3" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>562</v>
+        <v>569</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
       <c r="E13" s="17" t="n">
         <f aca="false">Assumptions!$C$12</f>
@@ -3659,14 +3680,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>564</v>
+        <v>571</v>
       </c>
       <c r="E15" s="18" t="n">
         <f aca="false">E13/E8</f>
         <v>0.0177100935790434</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
     </row>
   </sheetData>
@@ -3694,199 +3715,199 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>566</v>
+        <v>573</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>567</v>
+        <v>574</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>568</v>
+        <v>575</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>569</v>
+        <v>576</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>573</v>
+        <v>580</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>574</v>
+        <v>581</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>575</v>
+        <v>582</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>576</v>
+        <v>583</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>578</v>
+        <v>585</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>579</v>
+        <v>586</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>580</v>
+        <v>587</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>581</v>
+        <v>588</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>582</v>
+        <v>589</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>584</v>
+        <v>591</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>585</v>
+        <v>592</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>586</v>
+        <v>593</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>587</v>
+        <v>594</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>588</v>
+        <v>595</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>589</v>
+        <v>596</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>590</v>
+        <v>597</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>591</v>
+        <v>598</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>592</v>
+        <v>599</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>593</v>
+        <v>600</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>594</v>
+        <v>601</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>595</v>
+        <v>602</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>596</v>
+        <v>603</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>597</v>
+        <v>604</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>539</v>
+        <v>546</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>598</v>
+        <v>605</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>543</v>
+        <v>550</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>599</v>
+        <v>606</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>600</v>
+        <v>607</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>601</v>
+        <v>608</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>602</v>
+        <v>609</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>603</v>
+        <v>610</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>559</v>
+        <v>566</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>604</v>
+        <v>611</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>605</v>
+        <v>612</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>607</v>
+        <v>614</v>
       </c>
     </row>
   </sheetData>
@@ -5135,7 +5156,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
@@ -5479,6 +5500,74 @@
       </c>
       <c r="D27" s="16" t="s">
         <v>288</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
+        <v>293</v>
+      </c>
+      <c r="B32" s="18" t="n">
+        <f aca="false">B27</f>
+        <v>0.0025</v>
+      </c>
+      <c r="C32" s="22" t="n">
+        <f aca="false">E10*B32</f>
+        <v>2450</v>
+      </c>
+      <c r="D32" s="14" t="n">
+        <f aca="false">C32*E8</f>
+        <v>7519285.31073446</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="s">
+        <v>294</v>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C33" s="22" t="n">
+        <f aca="false">E10*B33</f>
+        <v>4900</v>
+      </c>
+      <c r="D33" s="14" t="n">
+        <f aca="false">C33*E8</f>
+        <v>15038570.6214689</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>295</v>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C34" s="22" t="n">
+        <f aca="false">E10*B34</f>
+        <v>9800</v>
+      </c>
+      <c r="D34" s="14" t="n">
+        <f aca="false">C34*E8</f>
+        <v>30077141.2429379</v>
       </c>
     </row>
   </sheetData>
@@ -5508,149 +5597,149 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="Y3" s="2" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="Z3" s="2" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="AA3" s="2" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="AB3" s="2" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="AC3" s="2" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="AD3" s="2" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="AE3" s="2" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="AF3" s="2" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="AG3" s="2" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="AH3" s="2" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="AI3" s="2" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="AJ3" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="AK3" s="2" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="AL3" s="2" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="AM3" s="2" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="AN3" s="2" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="AO3" s="2" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="AP3" s="2" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="AQ3" s="2" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="AR3" s="2" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>30000</v>
@@ -5783,7 +5872,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>239</v>
@@ -5917,7 +6006,7 @@
         <v>0</v>
       </c>
       <c r="AW5" s="16" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="AX5" s="22" t="n">
         <f aca="false">SUM(O21:AM21)+SUM(O25:AM25)</f>
@@ -5926,10 +6015,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>25000</v>
@@ -6060,7 +6149,7 @@
         <v>180000</v>
       </c>
       <c r="AW6" s="16" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="AX6" s="22" t="n">
         <f aca="false">SUM(O34:AM34)</f>
@@ -6069,10 +6158,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>8000</v>
@@ -6205,10 +6294,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>25000</v>
@@ -6341,10 +6430,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>342</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>335</v>
       </c>
       <c r="D9" s="4" t="n">
         <v>0</v>
@@ -6477,7 +6566,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>239</v>
@@ -6614,7 +6703,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>239</v>
@@ -6750,7 +6839,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>239</v>
@@ -6886,10 +6975,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>0</v>
@@ -7022,10 +7111,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>0</v>
@@ -7158,10 +7247,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D15" s="22" t="n">
         <f aca="false">D37*5*Assumptions!$C$27</f>
@@ -7330,10 +7419,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0</v>
@@ -7466,10 +7555,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>0</v>
@@ -7602,7 +7691,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>239</v>
@@ -7738,7 +7827,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>239</v>
@@ -7875,7 +7964,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>239</v>
@@ -8033,7 +8122,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>239</v>
@@ -8169,10 +8258,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>0</v>
@@ -8305,10 +8394,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>0</v>
@@ -8441,7 +8530,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>239</v>
@@ -8577,10 +8666,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D25" s="4" t="n">
         <v>0</v>
@@ -8713,7 +8802,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>239</v>
@@ -8850,10 +8939,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D27" s="22" t="n">
         <f aca="false">D39*Assumptions!$C$27</f>
@@ -9022,10 +9111,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D28" s="22" t="n">
         <f aca="false">D39*Assumptions!$C$33</f>
@@ -9194,10 +9283,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D29" s="22" t="n">
         <f aca="false">D41*Assumptions!$C$28</f>
@@ -9366,7 +9455,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="D30" s="23" t="n">
         <f aca="false">SUM(D4:D29)</f>
@@ -9535,7 +9624,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="D31" s="22" t="n">
         <f aca="false">D30*Assumptions!$C$35</f>
@@ -9704,7 +9793,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="D32" s="23" t="n">
         <f aca="false">D30+D31</f>
@@ -9873,7 +9962,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>239</v>
@@ -10009,7 +10098,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>239</v>
@@ -10161,7 +10250,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>239</v>
@@ -10333,10 +10422,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D37" s="4" t="n">
         <v>0</v>
@@ -10469,10 +10558,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D38" s="22" t="n">
         <f aca="false">D37*('Unit Economics'!$E$7-'Unit Economics'!$E$10-Assumptions!$C$29)</f>
@@ -10641,10 +10730,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D39" s="4" t="n">
         <v>0</v>
@@ -10777,10 +10866,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D40" s="22" t="n">
         <f aca="false">D39*('Unit Economics'!$C$7-'Unit Economics'!$C$9-'Unit Economics'!$C$10)</f>
@@ -10949,10 +11038,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D41" s="22" t="n">
         <f aca="false">D39*Assumptions!$C$34</f>
@@ -11101,10 +11190,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D42" s="22" t="n">
         <f aca="false">D41*'Unit Economics'!$D$7</f>
@@ -11273,7 +11362,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="B43" s="3"/>
       <c r="D43" s="22" t="n">
@@ -11443,7 +11532,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="9" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="B45" s="3"/>
       <c r="D45" s="22" t="n">
@@ -11613,7 +11702,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="B46" s="3"/>
       <c r="D46" s="22" t="n">
@@ -11763,7 +11852,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="D47" s="22" t="n">
         <f aca="false">IF(AND(1&gt;=13,MIN(D45:AM45)&gt;=0),1,0)</f>
@@ -11912,7 +12001,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="D48" s="22" t="n">
         <f aca="false">D46+'Funding Scenarios'!$C$7+IF(1&gt;=Assumptions!$C$43,'Funding Scenarios'!$C$6,0)</f>
@@ -12061,7 +12150,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="D49" s="22" t="n">
         <f aca="false">D46+'Funding Scenarios'!$D$7</f>
@@ -12210,7 +12299,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="D50" s="22" t="n">
         <f aca="false">D46+'Funding Scenarios'!$E$7</f>
@@ -12359,7 +12448,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="D51" s="22" t="n">
         <f aca="false">D46+'Funding Scenarios'!$F$7</f>
@@ -12508,7 +12597,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="D52" s="22" t="n">
         <f aca="false">IF(D48&lt;0,1,0)</f>
@@ -12657,7 +12746,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="D53" s="22" t="n">
         <f aca="false">IF(D49&lt;0,1,0)</f>
@@ -12806,7 +12895,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="D54" s="22" t="n">
         <f aca="false">IF(D50&lt;0,1,0)</f>
@@ -12955,7 +13044,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="D55" s="22" t="n">
         <f aca="false">IF(D51&lt;0,1,0)</f>
@@ -13104,12 +13193,12 @@
     </row>
     <row r="59" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="D60" s="15" t="n">
         <f aca="false">AN32</f>
@@ -13118,7 +13207,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="D61" s="15" t="n">
         <f aca="false">AN43</f>
@@ -13127,7 +13216,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="9" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="D62" s="15" t="n">
         <f aca="false">AN32/12</f>
@@ -13136,7 +13225,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="D63" s="15" t="n">
         <f aca="false">-AN45/12</f>
@@ -13145,7 +13234,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="9" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="D64" s="15" t="n">
         <f aca="false">AO32</f>
@@ -13154,7 +13243,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="9" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="D65" s="15" t="n">
         <f aca="false">-MIN(D46:I46)</f>
@@ -13163,7 +13252,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="9" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="D66" s="15" t="n">
         <f aca="false">-MIN(D46:AM46)</f>
@@ -13172,7 +13261,7 @@
     </row>
     <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="9" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="D67" s="24" t="str">
         <f aca="false">INDEX($D$3:$AM$3,MATCH(-D66,D46:AM46,0))</f>
@@ -13182,7 +13271,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="9" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="D68" s="15" t="n">
         <f aca="false">D66*(1+Assumptions!$C$36)</f>
@@ -13191,7 +13280,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="9" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="D69" s="15" t="n">
         <f aca="false">D65*(1+Assumptions!$C$36)</f>
@@ -13200,7 +13289,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="9" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="D70" s="15" t="n">
         <f aca="false">D68-D69</f>
@@ -13209,7 +13298,7 @@
     </row>
     <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="9" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="D71" s="24" t="str">
         <f aca="false">IFERROR(INDEX($D$3:$AM$3,MATCH(1,D47:AM47,0)),"Not within 36 months")</f>
@@ -13219,7 +13308,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="9" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="D72" s="15" t="n">
         <f aca="false">AQ43</f>
@@ -13228,7 +13317,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="9" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="D73" s="15" t="n">
         <f aca="false">AQ45</f>
@@ -13237,7 +13326,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="9" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="D74" s="15" t="n">
         <f aca="false">AR43</f>
@@ -13246,7 +13335,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="9" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="D75" s="15" t="n">
         <f aca="false">AR45</f>
@@ -13255,7 +13344,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="9" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="D76" s="25" t="n">
         <f aca="false">IF(D74=0,0,D75/D74)</f>
@@ -13264,7 +13353,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="9" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="D77" s="15" t="n">
         <f aca="false">AM45</f>
@@ -13273,7 +13362,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="9" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="D78" s="15" t="n">
         <f aca="false">SUMIF($B$4:$B$29,"Shared",$AN$4:$AN$29)</f>
@@ -13282,7 +13371,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="9" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="D79" s="15" t="n">
         <f aca="false">SUMIF($B$4:$B$29,"TremoSense",$AN$4:$AN$29)</f>
@@ -13291,7 +13380,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="9" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="D80" s="15" t="n">
         <f aca="false">SUMIF($B$4:$B$29,"ParkinSense",$AN$4:$AN$29)</f>
@@ -13300,7 +13389,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="9" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="C81" s="14" t="n">
         <f aca="false">D81</f>
@@ -13313,7 +13402,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="9" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="D82" s="15" t="n">
         <f aca="false">(SUM(J32:O32)-SUM(J19:O19)*(1+Assumptions!$C$35))/6</f>
@@ -13349,128 +13438,128 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>158</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="B4" s="26" t="n">
         <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>1500000</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="B5" s="26" t="n">
         <v>14.5</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>2000000</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="B6" s="26" t="n">
         <v>15.5</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>1250000</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="B7" s="27" t="n">
         <f aca="false">SUM(B4:B6)</f>
         <v>34</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>1000000</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="B8" s="17" t="n">
         <f aca="false">Assumptions!$C$39</f>
         <v>125000</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>250000</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>225000</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="F9" s="15" t="n">
         <f aca="false">SUM(F4:F8)</f>
@@ -13479,24 +13568,24 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="B10" s="15" t="n">
         <f aca="false">B7*B8+B9</f>
         <v>4475000</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="F10" s="15" t="n">
         <f aca="false">Assumptions!$C$44</f>
         <v>7500000</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="H10" s="18" t="n">
         <f aca="false">F10/F9-1</f>
@@ -13505,24 +13594,24 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13615,23 +13704,23 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>241</v>
@@ -13651,7 +13740,7 @@
         <v>0.759783159507286</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13668,7 +13757,7 @@
         <v>0.800922523811424</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13685,7 +13774,7 @@
         <v>0.827072886275294</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13702,7 +13791,7 @@
         <v>0.85488150416785</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
     </row>
   </sheetData>
@@ -13732,7 +13821,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13741,21 +13830,21 @@
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="C4" s="28" t="n">
         <f aca="false">Forecast!$D$68</f>
@@ -13776,24 +13865,24 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="C6" s="28" t="n">
         <f aca="false">Assumptions!$C$37</f>
@@ -13811,7 +13900,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">C4-C6</f>
@@ -13832,7 +13921,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
       <c r="C8" s="28" t="n">
         <f aca="false">Valuation!$F$10</f>
@@ -13853,7 +13942,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C8+C7</f>
@@ -13874,7 +13963,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="C10" s="31" t="n">
         <f aca="false">C7/C9</f>
@@ -13895,7 +13984,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="C11" s="31" t="n">
         <f aca="false">Assumptions!$C$38</f>
@@ -13916,7 +14005,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
       <c r="C12" s="31" t="n">
         <f aca="false">1-C10-C11</f>
@@ -13937,58 +14026,58 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="F13" s="29" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="E14" s="29" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="F14" s="29" t="s">
-        <v>481</v>
+        <v>488</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="D15" s="29" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
       <c r="E15" s="29" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
       <c r="F15" s="29" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
       <c r="C16" s="32" t="str">
         <f aca="false">IFERROR(INDEX(Forecast!$D$3:$AM$3,MATCH(1,Forecast!$D$52:$AM$52,0)),"Never — reaches break-even "&amp;Forecast!$D$71)</f>
@@ -14013,12 +14102,12 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
       <c r="F18" s="14" t="n">
         <f aca="false">Forecast!$D$70</f>
@@ -14027,7 +14116,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="F19" s="11" t="n">
         <v>0</v>
@@ -14035,7 +14124,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
       <c r="F20" s="14" t="n">
         <f aca="false">F18-F19</f>
@@ -14044,7 +14133,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
       <c r="F21" s="14" t="n">
         <f aca="false">F9+Forecast!$D$64</f>
@@ -14053,7 +14142,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>493</v>
+        <v>500</v>
       </c>
       <c r="F22" s="18" t="n">
         <f aca="false">F20/(F21+F20)</f>
@@ -14062,7 +14151,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
       <c r="F23" s="18" t="n">
         <f aca="false">F12*(1-F22)</f>
@@ -14071,7 +14160,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>495</v>
+        <v>502</v>
       </c>
       <c r="F24" s="18" t="n">
         <f aca="false">1-F23-F11*(1-F22)</f>
@@ -14083,7 +14172,7 @@
         <v>202</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
     </row>
   </sheetData>
@@ -14112,26 +14201,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>501</v>
+        <v>508</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>502</v>
+        <v>509</v>
       </c>
       <c r="B4" s="17" t="n">
         <f aca="false">Forecast!AO4+Forecast!AO5+Forecast!AO16+Forecast!AO23+Forecast!AO24+Forecast!AO25</f>
@@ -14142,12 +14231,12 @@
         <v>720000</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>503</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">Forecast!AO10+Forecast!AO11+Forecast!AO13+Forecast!AO14+Forecast!AO22</f>
@@ -14158,12 +14247,12 @@
         <v>425000</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>506</v>
+        <v>513</v>
       </c>
       <c r="B6" s="17" t="n">
         <f aca="false">Forecast!AO12+Forecast!AO17+Forecast!AO18</f>
@@ -14174,12 +14263,12 @@
         <v>630000</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>507</v>
+        <v>514</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">Forecast!AO15+Forecast!AO19+Forecast!AO20+Forecast!AO26+Forecast!AO27</f>
@@ -14190,12 +14279,12 @@
         <v>2237360.7</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="B8" s="17" t="n">
         <f aca="false">Forecast!AO6+Forecast!AO7+Forecast!AO9</f>
@@ -14206,12 +14295,12 @@
         <v>341000</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">Forecast!AO21+Forecast!AO8+Forecast!AO28+Forecast!AO29</f>
@@ -14222,12 +14311,12 @@
         <v>459000</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">Forecast!AO31</f>
@@ -14240,7 +14329,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B11" s="15" t="n">
         <f aca="false">SUM(B4:B10)</f>
@@ -14253,7 +14342,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>515</v>
+        <v>522</v>
       </c>
       <c r="B12" s="14" t="n">
         <f aca="false">B11-Forecast!AO32</f>

</xml_diff>